<commit_message>
Name the project Lemmata
Function prefix LEMMA., Python package lemmata, CLI lemma. Each module is a
lemma: proven once, cited everywhere. The name is free on PyPI and npm.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/phase0.xlsx
+++ b/examples/phase0.xlsx
@@ -10,16 +10,16 @@
     <sheet name="Demo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="AF.CAGR" comment="cagr@0.1.0 sha256:36adfaaf1d88dc4dc61c4d9b729247767fe6c66046531556a968d95f3ab5b9cb">_xlfn.LAMBDA(_xlpm.start_value, _xlpm.end_value, _xlpm.years,
+    <definedName name="LEMMA.CAGR" comment="cagr@0.1.0 sha256:8cc95aaee97a25818aab2294a3b5737408d7d642b461c9cbb0f3221f049a100a">_xlfn.LAMBDA(_xlpm.start_value, _xlpm.end_value, _xlpm.years,
   IF(NOT(AND(ISNUMBER(_xlpm.start_value), ISNUMBER(_xlpm.end_value), ISNUMBER(_xlpm.years))), #VALUE!,
   IF(OR(_xlpm.start_value &lt;= 0, _xlpm.end_value &lt; 0, _xlpm.years &lt;= 0), #NUM!,
   (_xlpm.end_value / _xlpm.start_value) ^ (1 / _xlpm.years) - 1)))</definedName>
-    <definedName name="AF.LOAN_PAYMENT" comment="loan_payment@0.1.0 sha256:b5b17907788068d0d15f85446b556796c736162702069bd7667ee6ec31f28ff8">_xlfn.LAMBDA(_xlpm.principal, _xlpm.rate, _xlpm.periods,
+    <definedName name="LEMMA.LOAN_PAYMENT" comment="loan_payment@0.1.0 sha256:4bfe72dc102fce277814f695325b282fe6b01423a3c09f2edae22f64fde891aa">_xlfn.LAMBDA(_xlpm.principal, _xlpm.rate, _xlpm.periods,
   IF(NOT(AND(ISNUMBER(_xlpm.principal), ISNUMBER(_xlpm.rate), ISNUMBER(_xlpm.periods))), #VALUE!,
   IF(OR(_xlpm.principal &lt; 0, _xlpm.rate &lt; 0, _xlpm.periods &lt;= 0, _xlpm.periods &lt;&gt; INT(_xlpm.periods)), #NUM!,
   IF(_xlpm.rate = 0, _xlpm.principal / _xlpm.periods,
   _xlpm.principal * _xlpm.rate / (1 - (1 + _xlpm.rate) ^ (-_xlpm.periods))))))</definedName>
-    <definedName name="AF.NPV" comment="npv@0.1.0 sha256:8ee9e62933f26d4f453d4eb1a4e1554477d31803693c907b0ba1244e6cceb982">_xlfn.LAMBDA(_xlpm.rate, _xlpm.cashflows, _xlpm.first_period,
+    <definedName name="LEMMA.NPV" comment="npv@0.1.0 sha256:25f1aa18c949a8b22c29371a24c27577a0df9d85e3174c9ea3a8809f6ad58838">_xlfn.LAMBDA(_xlpm.rate, _xlpm.cashflows, _xlpm.first_period,
   IF(NOT(AND(ISNUMBER(_xlpm.rate), ISNUMBER(_xlpm.first_period))), #VALUE!,
   IF(OR(_xlpm.rate &lt;= -1, _xlpm.first_period &lt; 0, _xlpm.first_period &lt;&gt; INT(_xlpm.first_period)), #NUM!,
   _xlfn.LET(_xlpm.r, ROWS(_xlpm.cashflows), _xlpm.c, COLUMNS(_xlpm.cashflows),
@@ -457,11 +457,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AF.CAGR(100, 200, 10)</t>
+          <t>LEMMA.CAGR(100, 200, 10)</t>
         </is>
       </c>
       <c r="B2">
-        <f>AF.CAGR(E2, F2, G2)</f>
+        <f>LEMMA.CAGR(E2, F2, G2)</f>
         <v/>
       </c>
       <c r="E2" t="n">
@@ -477,11 +477,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AF.LOAN_PAYMENT(200000, 5%/12, 360)</t>
+          <t>LEMMA.LOAN_PAYMENT(200000, 5%/12, 360)</t>
         </is>
       </c>
       <c r="B3">
-        <f>AF.LOAN_PAYMENT(E3, F3/12, G3)</f>
+        <f>LEMMA.LOAN_PAYMENT(E3, F3/12, G3)</f>
         <v/>
       </c>
       <c r="E3" t="n">
@@ -497,11 +497,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AF.NPV(8%, E4:E9, first_period 0)</t>
+          <t>LEMMA.NPV(8%, E4:E9, first_period 0)</t>
         </is>
       </c>
       <c r="B4">
-        <f>AF.NPV(F4, E4:E9, G4)</f>
+        <f>LEMMA.NPV(F4, E4:E9, G4)</f>
         <v/>
       </c>
       <c r="E4" t="n">

</xml_diff>

<commit_message>
loan_payment 0.2.0 and npv 0.2.0 from AI review findings; dependents re-pinned
loan_payment rejects nonzero rates below 1e-6 per period, where its closed
form loses precision. npv reports a bad cashflow cell as #VALUE! before any
domain error. Both old hashes carry a low-severity advisory. The four loan
modules that pin loan_payment move to 0.1.1 with the new hash.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/phase0.xlsx
+++ b/examples/phase0.xlsx
@@ -14,17 +14,17 @@
   IF(NOT(AND(ISNUMBER(_xlpm.start_value), ISNUMBER(_xlpm.end_value), ISNUMBER(_xlpm.years))), #VALUE!,
   IF(OR(_xlpm.start_value &lt;= 0, _xlpm.end_value &lt; 0, _xlpm.years &lt;= 0), #NUM!,
   (_xlpm.end_value / _xlpm.start_value) ^ (1 / _xlpm.years) - 1)))</definedName>
-    <definedName name="LEMMA.LOAN_PAYMENT" comment="loan_payment@0.1.0 sha256:4bfe72dc102fce277814f695325b282fe6b01423a3c09f2edae22f64fde891aa">_xlfn.LAMBDA(_xlpm.principal, _xlpm.rate, _xlpm.periods,
+    <definedName name="LEMMA.LOAN_PAYMENT" comment="loan_payment@0.2.0 sha256:36280cefe512d0393c8d606a94f1aeecf251af9e1292a68ebc9e5424961a189b">_xlfn.LAMBDA(_xlpm.principal, _xlpm.rate, _xlpm.periods,
   IF(NOT(AND(ISNUMBER(_xlpm.principal), ISNUMBER(_xlpm.rate), ISNUMBER(_xlpm.periods))), #VALUE!,
-  IF(OR(_xlpm.principal &lt; 0, _xlpm.rate &lt; 0, _xlpm.periods &lt;= 0, _xlpm.periods &lt;&gt; INT(_xlpm.periods)), #NUM!,
+  IF(OR(_xlpm.principal &lt; 0, _xlpm.rate &lt; 0, AND(_xlpm.rate &lt;&gt; 0, _xlpm.rate &lt; 0.000001), _xlpm.periods &lt;= 0, _xlpm.periods &lt;&gt; INT(_xlpm.periods)), #NUM!,
   IF(_xlpm.rate = 0, _xlpm.principal / _xlpm.periods,
   _xlpm.principal * _xlpm.rate / (1 - (1 + _xlpm.rate) ^ (-_xlpm.periods))))))</definedName>
-    <definedName name="LEMMA.NPV" comment="npv@0.1.0 sha256:25f1aa18c949a8b22c29371a24c27577a0df9d85e3174c9ea3a8809f6ad58838">_xlfn.LAMBDA(_xlpm.rate, _xlpm.cashflows, _xlpm.first_period,
+    <definedName name="LEMMA.NPV" comment="npv@0.2.0 sha256:62b1cd6d163cf4e016181baa98f9ac6cca297dc6af0351308c0ad02471afc586">_xlfn.LAMBDA(_xlpm.rate, _xlpm.cashflows, _xlpm.first_period,
   IF(NOT(AND(ISNUMBER(_xlpm.rate), ISNUMBER(_xlpm.first_period))), #VALUE!,
-  IF(OR(_xlpm.rate &lt;= -1, _xlpm.first_period &lt; 0, _xlpm.first_period &lt;&gt; INT(_xlpm.first_period)), #NUM!,
   _xlfn.LET(_xlpm.r, ROWS(_xlpm.cashflows), _xlpm.c, COLUMNS(_xlpm.cashflows),
     IF(AND(_xlpm.r &gt; 1, _xlpm.c &gt; 1), #VALUE!,
     IF(COUNT(_xlpm.cashflows) &lt;&gt; _xlpm.r * _xlpm.c, #VALUE!,
+    IF(OR(_xlpm.rate &lt;= -1, _xlpm.first_period &lt; 0, _xlpm.first_period &lt;&gt; INT(_xlpm.first_period)), #NUM!,
     SUMPRODUCT(_xlpm.cashflows / (1 + _xlpm.rate) ^ (_xlpm.first_period + _xlfn.SEQUENCE(_xlpm.r, _xlpm.c) - 1))))))))</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>